<commit_message>
Trabajo pendiente: armonización, Mincer y Gini
Cambios que ya estaban en el árbol de trabajo, sin relación con la
extensión de empleo_pleno_rama.do:

- empleo_adecuado_serie.do: documentación de la adaptación multi-año
  (renombres p##, códigos de p21/p25/p27/p28/p32/p34 por período).
- armonizacion_empleo adecuado.do: rutas portables, corrección del
  rename del CSV de salarios y bloque urbano/nacional; se advierte en
  el encabezado que el ingreso y las horas de los 90 no se limpian bien
  y que la versión correcta es la del paper de Íconos.
- educ_ingrl_hora.do / _fig.do: controles por rama de actividad en la
  regresión y notas al pie acordes.
- gini_decomp5.do: se quita la definición local de $gd y $gh_root; la
  raíz la fija el master.
- gini_decomposition.xlsx: salida regenerada.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dashboards/data/Data final/desigualdad/gini_decomposition.xlsx
+++ b/Dashboards/data/Data final/desigualdad/gini_decomposition.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <workbookPr/>
   <bookViews>
     <workbookView activeTab="0"/>
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="17" uniqueCount="17">
   <si>
     <t>slaboral</t>
   </si>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -244,10 +244,10 @@
         <v>0.75429217680282479</v>
       </c>
       <c r="I3" s="1">
-        <v>0.95194766651444362</v>
+        <v>0.95194766651444363</v>
       </c>
       <c r="J3" s="1">
-        <v>0.73375117507014342</v>
+        <v>0.73375117507014343</v>
       </c>
       <c r="K3" s="1">
         <v>0.66097397909885669</v>
@@ -477,7 +477,7 @@
         <v>-0.0001102270867625</v>
       </c>
       <c r="P7" s="1">
-        <v>-0.031185044427598198</v>
+        <v>-0.031185044427598199</v>
       </c>
       <c r="Q7" s="1">
         <v>2011</v>
@@ -500,7 +500,7 @@
         <v>0.53141866575384633</v>
       </c>
       <c r="F8" s="1">
-        <v>0.91971154305627389</v>
+        <v>0.9197115430562739</v>
       </c>
       <c r="G8" s="1">
         <v>0.98401130653132307</v>
@@ -509,7 +509,7 @@
         <v>0.77463588021538399</v>
       </c>
       <c r="I8" s="1">
-        <v>0.9363005277007389</v>
+        <v>0.93630052770073891</v>
       </c>
       <c r="J8" s="1">
         <v>0.64337824094114437</v>
@@ -618,7 +618,7 @@
         <v>0.92538183041701216</v>
       </c>
       <c r="J10" s="1">
-        <v>0.57802712932923916</v>
+        <v>0.57802712932923917</v>
       </c>
       <c r="K10" s="1">
         <v>0.49262858230414758</v>
@@ -680,7 +680,7 @@
         <v>-0.3121255338443033</v>
       </c>
       <c r="M11" s="1">
-        <v>0.00049913281635660005</v>
+        <v>0.00049913281635660006</v>
       </c>
       <c r="N11" s="1">
         <v>0.025702756408549399</v>
@@ -730,7 +730,7 @@
         <v>0.41536560745237261</v>
       </c>
       <c r="L12" s="1">
-        <v>-0.32294752797140241</v>
+        <v>-0.32294752797140242</v>
       </c>
       <c r="M12" s="1">
         <v>0.029985990470625199</v>
@@ -777,7 +777,7 @@
         <v>0.90866866567465843</v>
       </c>
       <c r="J13" s="1">
-        <v>0.59074717444760227</v>
+        <v>0.59074717444760228</v>
       </c>
       <c r="K13" s="1">
         <v>0.48290553645140061</v>

</xml_diff>

<commit_message>
Corregir la homologación de ramas y llevarla a las copias del Boletín 1
En los códigos viejos que se reparten entre varios nuevos se elige primero la
sección a la que apunta la mayoría de los destinos (antes ganaba el código
menor: la construcción de los 90 terminaba en minas). Los códigos que no están
en la correspondencia se emparejan por grupo de 3 dígitos o división de 2.
Las copias del Boletín 1 se reemplazan por las del Boletín 3, que son las que
usa el paper de Íconos (incluye isic3_31.do, que faltaba). También van los
cambios pendientes de adec.do, iess_issfa_isspol.do, el log del boletín 3 y
gini_decomposition.xlsx del dashboard.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dashboards/data/Data final/desigualdad/gini_decomposition.xlsx
+++ b/Dashboards/data/Data final/desigualdad/gini_decomposition.xlsx
@@ -167,52 +167,52 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>89.480968899649397</v>
+        <v>89.48095941683701</v>
       </c>
       <c r="B2" s="1">
-        <v>0.24823623403464001</v>
+        <v>0.24823645781737999</v>
       </c>
       <c r="C2" s="1">
-        <v>9.3060989860159591</v>
+        <v>9.3061073753809307</v>
       </c>
       <c r="D2" s="1">
-        <v>0.96469588030000009</v>
+        <v>0.96469674996470001</v>
       </c>
       <c r="E2" s="1">
-        <v>0.59447178814201596</v>
+        <v>0.56766737870934747</v>
       </c>
       <c r="F2" s="1">
-        <v>0.9991763803390038</v>
+        <v>0.99912193800383675</v>
       </c>
       <c r="G2" s="1">
-        <v>0.99089001036765789</v>
+        <v>0.99028782815606797</v>
       </c>
       <c r="H2" s="1">
-        <v>0.79680469261046849</v>
+        <v>0.78337321743630739</v>
       </c>
       <c r="I2" s="1">
-        <v>0.98373233338987132</v>
+        <v>0.98183816733612128</v>
       </c>
       <c r="J2" s="1">
-        <v>0.83591251478564299</v>
+        <v>0.82505665524652794</v>
       </c>
       <c r="K2" s="1">
-        <v>0.89291892722410682</v>
+        <v>0.88577130958406025</v>
       </c>
       <c r="L2" s="1">
-        <v>-0.1920524874828862</v>
+        <v>-0.2926382694376421</v>
       </c>
       <c r="M2" s="1">
-        <v>-0.031617704557796701</v>
+        <v>-0.035219596450556799</v>
       </c>
       <c r="N2" s="1">
-        <v>0.00093772097689240005</v>
+        <v>0.0010445480833004999</v>
       </c>
       <c r="O2" s="1">
-        <v>0.0427621207072853</v>
+        <v>0.047633705470166703</v>
       </c>
       <c r="P2" s="1">
-        <v>-0.012082137126363199</v>
+        <v>-0.0134586571028915</v>
       </c>
       <c r="Q2" s="1">
         <v>2001</v>
@@ -232,40 +232,40 @@
         <v>1.1749957088168399</v>
       </c>
       <c r="E3" s="1">
-        <v>0.58040887486662351</v>
+        <v>0.57892466866688774</v>
       </c>
       <c r="F3" s="1">
-        <v>0.94927902416577359</v>
+        <v>0.94909961048832414</v>
       </c>
       <c r="G3" s="1">
-        <v>0.97154227319774966</v>
+        <v>0.97144161059546186</v>
       </c>
       <c r="H3" s="1">
-        <v>0.75429217680282479</v>
+        <v>0.75342304241780744</v>
       </c>
       <c r="I3" s="1">
-        <v>0.95194766651444363</v>
+        <v>0.95165406359186422</v>
       </c>
       <c r="J3" s="1">
-        <v>0.73375117507014343</v>
+        <v>0.7327588731032767</v>
       </c>
       <c r="K3" s="1">
-        <v>0.66097397909885669</v>
+        <v>0.65973949847427671</v>
       </c>
       <c r="L3" s="1">
-        <v>-0.36010344654960469</v>
+        <v>-0.36648903596202148</v>
       </c>
       <c r="M3" s="1">
-        <v>-0.0095388033277474995</v>
+        <v>-0.0095993663608525005</v>
       </c>
       <c r="N3" s="1">
-        <v>0.021330324053373501</v>
+        <v>0.021465752898731101</v>
       </c>
       <c r="O3" s="1">
-        <v>0.0056710357601498004</v>
+        <v>0.0057070418622168001</v>
       </c>
       <c r="P3" s="1">
-        <v>-0.017462556485740601</v>
+        <v>-0.0175734284001118</v>
       </c>
       <c r="Q3" s="1">
         <v>2003</v>
@@ -273,7 +273,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>86.833009839686909</v>
+        <v>86.833009839686923</v>
       </c>
       <c r="B4" s="1">
         <v>9.2680375342012589</v>
@@ -285,40 +285,40 @@
         <v>0.79879905278272012</v>
       </c>
       <c r="E4" s="1">
-        <v>0.55964380964185523</v>
+        <v>0.55343209817574801</v>
       </c>
       <c r="F4" s="1">
-        <v>0.94656328638551512</v>
+        <v>0.94580950239442396</v>
       </c>
       <c r="G4" s="1">
-        <v>0.97774870407863235</v>
+        <v>0.97743482492116907</v>
       </c>
       <c r="H4" s="1">
-        <v>0.78052695097633273</v>
+        <v>0.77743104069968283</v>
       </c>
       <c r="I4" s="1">
-        <v>0.95588232734042022</v>
+        <v>0.95475783780348578</v>
       </c>
       <c r="J4" s="1">
-        <v>0.74339466132109777</v>
+        <v>0.73956756684555636</v>
       </c>
       <c r="K4" s="1">
-        <v>0.67073820756426417</v>
+        <v>0.66598637971655172</v>
       </c>
       <c r="L4" s="1">
-        <v>-0.38305038891667381</v>
+        <v>-0.40814516327124789</v>
       </c>
       <c r="M4" s="1">
-        <v>-0.020170633696055301</v>
+        <v>-0.0206962787186287</v>
       </c>
       <c r="N4" s="1">
-        <v>0.026398136603728101</v>
+        <v>0.0270860698298095</v>
       </c>
       <c r="O4" s="1">
-        <v>0.0061212043253248997</v>
+        <v>0.0062807223967034998</v>
       </c>
       <c r="P4" s="1">
-        <v>-0.0123487072329957</v>
+        <v>-0.0126705135078961</v>
       </c>
       <c r="Q4" s="1">
         <v>2005</v>
@@ -326,7 +326,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1">
-        <v>85.688927968079511</v>
+        <v>85.688927968079497</v>
       </c>
       <c r="B5" s="1">
         <v>9.7460581018909096</v>
@@ -338,40 +338,40 @@
         <v>1.5525669223724199</v>
       </c>
       <c r="E5" s="1">
-        <v>0.58863054633415257</v>
+        <v>0.58232838345702498</v>
       </c>
       <c r="F5" s="1">
-        <v>0.93032440464950095</v>
+        <v>0.92925697743403413</v>
       </c>
       <c r="G5" s="1">
-        <v>0.97602121708747425</v>
+        <v>0.9756538631330911</v>
       </c>
       <c r="H5" s="1">
-        <v>0.75956565618753713</v>
+        <v>0.75588221206580619</v>
       </c>
       <c r="I5" s="1">
-        <v>0.9498964894681784</v>
+        <v>0.94857836087621128</v>
       </c>
       <c r="J5" s="1">
-        <v>0.70697250426850666</v>
+        <v>0.70214158114912806</v>
       </c>
       <c r="K5" s="1">
-        <v>0.6450529809010449</v>
+        <v>0.63947951500531641</v>
       </c>
       <c r="L5" s="1">
-        <v>-0.38786317641835338</v>
+        <v>-0.41599190554180759</v>
       </c>
       <c r="M5" s="1">
-        <v>0.0023443156603260998</v>
+        <v>0.0024095163206241002</v>
       </c>
       <c r="N5" s="1">
-        <v>0.017495882480779101</v>
+        <v>0.017982482092406899</v>
       </c>
       <c r="O5" s="1">
-        <v>0.0038882623496321999</v>
+        <v>0.0039964036195184001</v>
       </c>
       <c r="P5" s="1">
-        <v>-0.023728460490765501</v>
+        <v>-0.0243884020325532</v>
       </c>
       <c r="Q5" s="1">
         <v>2007</v>
@@ -379,10 +379,10 @@
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <v>84.694858003146351</v>
+        <v>84.694858003146365</v>
       </c>
       <c r="B6" s="1">
-        <v>11.06434268598573</v>
+        <v>11.064342685985739</v>
       </c>
       <c r="C6" s="1">
         <v>1.87816264831776</v>
@@ -391,40 +391,40 @@
         <v>2.36263666255015</v>
       </c>
       <c r="E6" s="1">
-        <v>0.55113649340228998</v>
+        <v>0.54269994250177989</v>
       </c>
       <c r="F6" s="1">
-        <v>0.92470807630297192</v>
+        <v>0.92329293754179975</v>
       </c>
       <c r="G6" s="1">
-        <v>0.98071159660645346</v>
+        <v>0.980349064133615</v>
       </c>
       <c r="H6" s="1">
-        <v>0.75322805139021942</v>
+        <v>0.7485898839413978</v>
       </c>
       <c r="I6" s="1">
-        <v>0.93808843041571133</v>
+        <v>0.93594424334948734</v>
       </c>
       <c r="J6" s="1">
-        <v>0.69344073995142785</v>
+        <v>0.68720015127483847</v>
       </c>
       <c r="K6" s="1">
-        <v>0.56599467980179941</v>
+        <v>0.55767388239764359</v>
       </c>
       <c r="L6" s="1">
-        <v>-0.33484380543565012</v>
+        <v>-0.3683586438302649</v>
       </c>
       <c r="M6" s="1">
-        <v>0.0061307212533962003</v>
+        <v>0.0063592817406685999</v>
       </c>
       <c r="N6" s="1">
-        <v>0.027575982869121</v>
+        <v>0.028604047891428199</v>
       </c>
       <c r="O6" s="1">
-        <v>0.001528670361063</v>
+        <v>0.0015856609871559</v>
       </c>
       <c r="P6" s="1">
-        <v>-0.035235374483575603</v>
+        <v>-0.036548990619269903</v>
       </c>
       <c r="Q6" s="1">
         <v>2009</v>
@@ -432,52 +432,52 @@
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <v>85.481966211100598</v>
+        <v>85.481966211100627</v>
       </c>
       <c r="B7" s="1">
         <v>11.192253691238351</v>
       </c>
       <c r="C7" s="1">
-        <v>1.4583763892672199</v>
+        <v>1.4583763892672101</v>
       </c>
       <c r="D7" s="1">
         <v>1.86740370839379</v>
       </c>
       <c r="E7" s="1">
-        <v>0.52013465224501854</v>
+        <v>0.51420508947147381</v>
       </c>
       <c r="F7" s="1">
-        <v>0.91462830089478431</v>
+        <v>0.91357338652912912</v>
       </c>
       <c r="G7" s="1">
-        <v>0.98177442109251178</v>
+        <v>0.98154921267784434</v>
       </c>
       <c r="H7" s="1">
-        <v>0.81271584786116036</v>
+        <v>0.81040162962935203</v>
       </c>
       <c r="I7" s="1">
-        <v>0.92565879073766011</v>
+        <v>0.92387231742914955</v>
       </c>
       <c r="J7" s="1">
-        <v>0.65623474423320272</v>
+        <v>0.65158507753500217</v>
       </c>
       <c r="K7" s="1">
-        <v>0.48489814463290482</v>
+        <v>0.47841352783983948</v>
       </c>
       <c r="L7" s="1">
-        <v>-0.39543264853466159</v>
+        <v>-0.41670972016448221</v>
       </c>
       <c r="M7" s="1">
-        <v>0.0031739037060889001</v>
+        <v>0.0032567742473939001</v>
       </c>
       <c r="N7" s="1">
-        <v>0.028121367808295501</v>
+        <v>0.028855615973639001</v>
       </c>
       <c r="O7" s="1">
-        <v>-0.0001102270867625</v>
+        <v>-0.0001131051130651</v>
       </c>
       <c r="P7" s="1">
-        <v>-0.031185044427598199</v>
+        <v>-0.031999285107970198</v>
       </c>
       <c r="Q7" s="1">
         <v>2011</v>
@@ -488,49 +488,49 @@
         <v>86.6899212833343</v>
       </c>
       <c r="B8" s="1">
-        <v>9.8729959056215399</v>
+        <v>9.8729959056215311</v>
       </c>
       <c r="C8" s="1">
-        <v>1.05298745495754</v>
+        <v>1.05298745495753</v>
       </c>
       <c r="D8" s="1">
         <v>2.3840953560866298</v>
       </c>
       <c r="E8" s="1">
-        <v>0.53141866575384633</v>
+        <v>0.52890531586682188</v>
       </c>
       <c r="F8" s="1">
-        <v>0.9197115430562739</v>
+        <v>0.9192808964012914</v>
       </c>
       <c r="G8" s="1">
-        <v>0.98401130653132307</v>
+        <v>0.98392554728744353</v>
       </c>
       <c r="H8" s="1">
-        <v>0.77463588021538399</v>
+        <v>0.77342708497838719</v>
       </c>
       <c r="I8" s="1">
-        <v>0.93630052770073891</v>
+        <v>0.93565453759020412</v>
       </c>
       <c r="J8" s="1">
-        <v>0.64337824094114437</v>
+        <v>0.64129745421062789</v>
       </c>
       <c r="K8" s="1">
-        <v>0.42784957232665322</v>
+        <v>0.4247305681467014</v>
       </c>
       <c r="L8" s="1">
-        <v>-0.34591976482683512</v>
+        <v>-0.35525376406137271</v>
       </c>
       <c r="M8" s="1">
-        <v>0.017347007154057001</v>
+        <v>0.017538828913493301</v>
       </c>
       <c r="N8" s="1">
-        <v>0.021032166035045499</v>
+        <v>0.021264737974261001</v>
       </c>
       <c r="O8" s="1">
-        <v>-0.0014419038433813999</v>
+        <v>-0.0014578482959147999</v>
       </c>
       <c r="P8" s="1">
-        <v>-0.036937269345715298</v>
+        <v>-0.0373457185918281</v>
       </c>
       <c r="Q8" s="1">
         <v>2013</v>
@@ -538,10 +538,10 @@
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <v>86.104365759074852</v>
+        <v>86.104365759074838</v>
       </c>
       <c r="B9" s="1">
-        <v>11.952110391905601</v>
+        <v>11.95211039190561</v>
       </c>
       <c r="C9" s="1">
         <v>0.71941396446384998</v>
@@ -550,40 +550,40 @@
         <v>1.2241098845556999</v>
       </c>
       <c r="E9" s="1">
-        <v>0.52605055562709857</v>
+        <v>0.52098014158685857</v>
       </c>
       <c r="F9" s="1">
-        <v>0.85748463152096421</v>
+        <v>0.85595997117193767</v>
       </c>
       <c r="G9" s="1">
-        <v>0.98953484140262449</v>
+        <v>0.98942288286418201</v>
       </c>
       <c r="H9" s="1">
-        <v>0.87392434605994274</v>
+        <v>0.87257556134570413</v>
       </c>
       <c r="I9" s="1">
-        <v>0.93594927850458132</v>
+        <v>0.93463401047818251</v>
       </c>
       <c r="J9" s="1">
-        <v>0.56426764855904354</v>
+        <v>0.55882164706252802</v>
       </c>
       <c r="K9" s="1">
-        <v>0.448398221449544</v>
+        <v>0.44243398141615292</v>
       </c>
       <c r="L9" s="1">
-        <v>-0.33469024879354442</v>
+        <v>-0.35105422533270131</v>
       </c>
       <c r="M9" s="1">
-        <v>0.019629175971377099</v>
+        <v>0.020070500160420099</v>
       </c>
       <c r="N9" s="1">
-        <v>0.00061283649263230004</v>
+        <v>0.00062661494000820002</v>
       </c>
       <c r="O9" s="1">
-        <v>-0.0005630718920506</v>
+        <v>-0.00057573147829480004</v>
       </c>
       <c r="P9" s="1">
-        <v>-0.019678940571940098</v>
+        <v>-0.020121383622093099</v>
       </c>
       <c r="Q9" s="1">
         <v>2015</v>
@@ -591,7 +591,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1">
-        <v>84.349828847937886</v>
+        <v>84.349828847937857</v>
       </c>
       <c r="B10" s="1">
         <v>13.575145216937129</v>
@@ -603,40 +603,40 @@
         <v>1.1866440811151799</v>
       </c>
       <c r="E10" s="1">
-        <v>0.50632850571127708</v>
+        <v>0.50387142391000628</v>
       </c>
       <c r="F10" s="1">
-        <v>0.84493192361532776</v>
+        <v>0.84416012505526905</v>
       </c>
       <c r="G10" s="1">
-        <v>0.98823735890763265</v>
+        <v>0.98817881436597155</v>
       </c>
       <c r="H10" s="1">
-        <v>0.87482546782402071</v>
+        <v>0.87420245420357623</v>
       </c>
       <c r="I10" s="1">
-        <v>0.92538183041701216</v>
+        <v>0.9246447643341057</v>
       </c>
       <c r="J10" s="1">
-        <v>0.57802712932923917</v>
+        <v>0.57553918154733386</v>
       </c>
       <c r="K10" s="1">
-        <v>0.49262858230414758</v>
+        <v>0.49007310502669799</v>
       </c>
       <c r="L10" s="1">
-        <v>-0.36194506295603168</v>
+        <v>-0.36969912252042703</v>
       </c>
       <c r="M10" s="1">
-        <v>0.011793499474987</v>
+        <v>0.0119212682061183</v>
       </c>
       <c r="N10" s="1">
-        <v>0.0077284842432014996</v>
+        <v>0.0078122133032457004</v>
       </c>
       <c r="O10" s="1">
-        <v>0.00047578176647989999</v>
+        <v>0.00048093630375149998</v>
       </c>
       <c r="P10" s="1">
-        <v>-0.019997765484637699</v>
+        <v>-0.020214417813114598</v>
       </c>
       <c r="Q10" s="1">
         <v>2017</v>
@@ -644,10 +644,10 @@
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <v>80.572585852026435</v>
+        <v>80.572585852026478</v>
       </c>
       <c r="B11" s="1">
-        <v>17.17863077418156</v>
+        <v>17.178630774181571</v>
       </c>
       <c r="C11" s="1">
         <v>0.59984857052927998</v>
@@ -656,40 +656,40 @@
         <v>1.6489348032626898</v>
       </c>
       <c r="E11" s="1">
-        <v>0.52584087785161082</v>
+        <v>0.52330152400681673</v>
       </c>
       <c r="F11" s="1">
-        <v>0.8414116597365241</v>
+        <v>0.84056234166424504</v>
       </c>
       <c r="G11" s="1">
-        <v>0.99051246743284127</v>
+        <v>0.99046165705890155</v>
       </c>
       <c r="H11" s="1">
-        <v>0.88550547552848902</v>
+        <v>0.88489230139062813</v>
       </c>
       <c r="I11" s="1">
-        <v>0.90695821816197364</v>
+        <v>0.90600602484099757</v>
       </c>
       <c r="J11" s="1">
-        <v>0.6512063861234525</v>
+        <v>0.64898411160208558</v>
       </c>
       <c r="K11" s="1">
-        <v>0.4691142544583316</v>
+        <v>0.46624372169413858</v>
       </c>
       <c r="L11" s="1">
-        <v>-0.3121255338443033</v>
+        <v>-0.32006669631710932</v>
       </c>
       <c r="M11" s="1">
-        <v>0.00049913281635660006</v>
+        <v>0.00050477444039890001</v>
       </c>
       <c r="N11" s="1">
-        <v>0.025702756408549399</v>
+        <v>0.025993270845927501</v>
       </c>
       <c r="O11" s="1">
-        <v>-0.00015048341776440001</v>
+        <v>-0.00015218430948030001</v>
       </c>
       <c r="P11" s="1">
-        <v>-0.026051405807126799</v>
+        <v>-0.026345860976859502</v>
       </c>
       <c r="Q11" s="1">
         <v>2019</v>
@@ -697,7 +697,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1">
-        <v>79.781416995946955</v>
+        <v>79.781416995946927</v>
       </c>
       <c r="B12" s="1">
         <v>16.847581034108412</v>
@@ -709,40 +709,40 @@
         <v>2.7621405740919602</v>
       </c>
       <c r="E12" s="1">
-        <v>0.54367122647984412</v>
+        <v>0.54127090823848478</v>
       </c>
       <c r="F12" s="1">
-        <v>0.82442999396936201</v>
+        <v>0.82350648462134468</v>
       </c>
       <c r="G12" s="1">
-        <v>0.99170828400055011</v>
+        <v>0.9916646690494012</v>
       </c>
       <c r="H12" s="1">
-        <v>0.8090895913927173</v>
+        <v>0.80808539055588202</v>
       </c>
       <c r="I12" s="1">
-        <v>0.90950365304997494</v>
+        <v>0.90862421078267053</v>
       </c>
       <c r="J12" s="1">
-        <v>0.62472925213937425</v>
+        <v>0.62233224867792558</v>
       </c>
       <c r="K12" s="1">
-        <v>0.41536560745237261</v>
+        <v>0.41226454515062311</v>
       </c>
       <c r="L12" s="1">
-        <v>-0.32294752797140242</v>
+        <v>-0.33155897899060233</v>
       </c>
       <c r="M12" s="1">
-        <v>0.029985990470625199</v>
+        <v>0.0303188866074811</v>
       </c>
       <c r="N12" s="1">
-        <v>0.013605824222656</v>
+        <v>0.0137568723038171</v>
       </c>
       <c r="O12" s="1">
-        <v>-0.00082582593171740004</v>
+        <v>-0.00083499402181729996</v>
       </c>
       <c r="P12" s="1">
-        <v>-0.042765988761565302</v>
+        <v>-0.043240764889464004</v>
       </c>
       <c r="Q12" s="1">
         <v>2021</v>
@@ -750,7 +750,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <v>80.101133299132741</v>
+        <v>80.101133299132727</v>
       </c>
       <c r="B13" s="1">
         <v>17.307855339711761</v>
@@ -762,40 +762,40 @@
         <v>2.05846843941928</v>
       </c>
       <c r="E13" s="1">
-        <v>0.51940908950109455</v>
+        <v>0.51836943049408368</v>
       </c>
       <c r="F13" s="1">
-        <v>0.81605005266722686</v>
+        <v>0.81565211501297141</v>
       </c>
       <c r="G13" s="1">
-        <v>0.99095560805041727</v>
+        <v>0.99093604237959898</v>
       </c>
       <c r="H13" s="1">
-        <v>0.82919779786109127</v>
+        <v>0.82882830263346119</v>
       </c>
       <c r="I13" s="1">
-        <v>0.90866866567465843</v>
+        <v>0.90828751579399847</v>
       </c>
       <c r="J13" s="1">
-        <v>0.59074717444760228</v>
+        <v>0.58966174378073222</v>
       </c>
       <c r="K13" s="1">
-        <v>0.48290553645140061</v>
+        <v>0.48177667763096499</v>
       </c>
       <c r="L13" s="1">
-        <v>-0.32847314078613782</v>
+        <v>-0.33194053781826322</v>
       </c>
       <c r="M13" s="1">
-        <v>0.0236537435218225</v>
+        <v>0.023765648754681699</v>
       </c>
       <c r="N13" s="1">
-        <v>0.0089273823324855003</v>
+        <v>0.0089696175413757993</v>
       </c>
       <c r="O13" s="1">
-        <v>0.0002335473822991</v>
+        <v>0.00023465228876669999</v>
       </c>
       <c r="P13" s="1">
-        <v>-0.032814673236616902</v>
+        <v>-0.032969918584839102</v>
       </c>
       <c r="Q13" s="1">
         <v>2023</v>
@@ -815,40 +815,40 @@
         <v>2.3188250225661799</v>
       </c>
       <c r="E14" s="1">
-        <v>0.53274673709590914</v>
+        <v>0.53076028696925981</v>
       </c>
       <c r="F14" s="1">
-        <v>0.82337662271585332</v>
+        <v>0.8226257375791971</v>
       </c>
       <c r="G14" s="1">
-        <v>0.99232437906602999</v>
+        <v>0.99229174743049842</v>
       </c>
       <c r="H14" s="1">
-        <v>0.7887134630014041</v>
+        <v>0.78781521316240311</v>
       </c>
       <c r="I14" s="1">
-        <v>0.90943486771752591</v>
+        <v>0.90870945038416806</v>
       </c>
       <c r="J14" s="1">
-        <v>0.62032075723022595</v>
+        <v>0.61835857253249471</v>
       </c>
       <c r="K14" s="1">
-        <v>0.53791537101929821</v>
+        <v>0.53593563417507772</v>
       </c>
       <c r="L14" s="1">
-        <v>-0.33385280600297218</v>
+        <v>-0.34105075668519053</v>
       </c>
       <c r="M14" s="1">
-        <v>0.021462985139933499</v>
+        <v>0.021657278710768699</v>
       </c>
       <c r="N14" s="1">
-        <v>0.013874593112782</v>
+        <v>0.014000192800891599</v>
       </c>
       <c r="O14" s="1">
-        <v>0.00079006493367780005</v>
+        <v>0.00079721699272949996</v>
       </c>
       <c r="P14" s="1">
-        <v>-0.0361276431864117</v>
+        <v>-0.036454688504398897</v>
       </c>
       <c r="Q14" s="1">
         <v>2025</v>

</xml_diff>